<commit_message>
separate stocker date with dc process date on import stocker manual
</commit_message>
<xml_diff>
--- a/public/assets/example/contoh-import-stocker-manual.xlsx
+++ b/public/assets/example/contoh-import-stocker-manual.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip_local_main\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828AE324-F57F-4BF7-AFBF-2A7E234EB4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BCFB8B-371A-4B85-861E-9E9767BB90C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
   <si>
     <t>act_costing_ws</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>tanggal</t>
+  </si>
+  <si>
+    <t>tanggal proses dc</t>
   </si>
 </sst>
 </file>
@@ -723,10 +726,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="29.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -737,20 +740,21 @@
     <col min="9" max="9" width="11.28515625" style="1" customWidth="1"/>
     <col min="10" max="10" width="17.42578125" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.28515625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="6.85546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.7109375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16" style="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="1" customWidth="1"/>
-    <col min="21" max="21" width="15.42578125" style="1" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="1"/>
+    <col min="12" max="12" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.85546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="16" style="1" customWidth="1"/>
+    <col min="20" max="20" width="15.140625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="12" style="1" customWidth="1"/>
+    <col min="22" max="22" width="15.42578125" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:22">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -784,39 +788,44 @@
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
-      <c r="A2" s="5"/>
+    <row r="2" spans="1:22">
+      <c r="A2" s="4">
+        <v>45919</v>
+      </c>
       <c r="B2" s="8" t="s">
         <v>16</v>
       </c>
@@ -847,26 +856,31 @@
       <c r="K2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="4">
+        <v>45919</v>
+      </c>
+      <c r="M2" s="9">
         <v>1</v>
       </c>
-      <c r="M2" s="9"/>
       <c r="N2" s="9"/>
-      <c r="R2" s="9">
+      <c r="O2" s="9"/>
+      <c r="S2" s="9">
         <v>1</v>
       </c>
-      <c r="S2" s="4">
-        <v>45919</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="T2" s="4">
+        <v>45919</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="V2" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
-      <c r="A3" s="5"/>
+    <row r="3" spans="1:22">
+      <c r="A3" s="4">
+        <v>45919</v>
+      </c>
       <c r="B3" s="8" t="s">
         <v>27</v>
       </c>
@@ -897,8 +911,8 @@
       <c r="K3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="9">
-        <v>3</v>
+      <c r="L3" s="4">
+        <v>45919</v>
       </c>
       <c r="M3" s="9">
         <v>3</v>
@@ -912,24 +926,29 @@
       <c r="P3" s="9">
         <v>3</v>
       </c>
-      <c r="Q3" s="4">
-        <v>45919</v>
-      </c>
-      <c r="R3" s="9">
+      <c r="Q3" s="9">
         <v>3</v>
       </c>
-      <c r="S3" s="4">
-        <v>45919</v>
-      </c>
-      <c r="T3" s="3" t="s">
+      <c r="R3" s="4">
+        <v>45919</v>
+      </c>
+      <c r="S3" s="9">
+        <v>3</v>
+      </c>
+      <c r="T3" s="4">
+        <v>45919</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U3" s="8" t="s">
+      <c r="V3" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
-      <c r="A4" s="5"/>
+    <row r="4" spans="1:22">
+      <c r="A4" s="4">
+        <v>45919</v>
+      </c>
       <c r="B4" s="8" t="s">
         <v>34</v>
       </c>
@@ -960,8 +979,8 @@
       <c r="K4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="9">
-        <v>1</v>
+      <c r="L4" s="4">
+        <v>45919</v>
       </c>
       <c r="M4" s="9">
         <v>1</v>
@@ -975,24 +994,29 @@
       <c r="P4" s="9">
         <v>1</v>
       </c>
-      <c r="Q4" s="4">
-        <v>45919</v>
-      </c>
-      <c r="R4" s="9">
+      <c r="Q4" s="9">
         <v>1</v>
       </c>
-      <c r="S4" s="4">
-        <v>45919</v>
-      </c>
-      <c r="T4" s="3" t="s">
+      <c r="R4" s="4">
+        <v>45919</v>
+      </c>
+      <c r="S4" s="9">
+        <v>1</v>
+      </c>
+      <c r="T4" s="4">
+        <v>45919</v>
+      </c>
+      <c r="U4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U4" s="8" t="s">
+      <c r="V4" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
-      <c r="A5" s="5"/>
+    <row r="5" spans="1:22">
+      <c r="A5" s="4">
+        <v>45919</v>
+      </c>
       <c r="B5" s="8" t="s">
         <v>37</v>
       </c>
@@ -1023,8 +1047,8 @@
       <c r="K5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="9">
-        <v>2</v>
+      <c r="L5" s="4">
+        <v>45919</v>
       </c>
       <c r="M5" s="9">
         <v>2</v>
@@ -1038,24 +1062,29 @@
       <c r="P5" s="9">
         <v>2</v>
       </c>
-      <c r="Q5" s="4">
-        <v>45919</v>
-      </c>
-      <c r="R5" s="9">
+      <c r="Q5" s="9">
         <v>2</v>
       </c>
-      <c r="S5" s="4">
-        <v>45919</v>
-      </c>
-      <c r="T5" s="3" t="s">
+      <c r="R5" s="4">
+        <v>45919</v>
+      </c>
+      <c r="S5" s="9">
+        <v>2</v>
+      </c>
+      <c r="T5" s="4">
+        <v>45919</v>
+      </c>
+      <c r="U5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U5" s="8" t="s">
+      <c r="V5" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
-      <c r="A6" s="5"/>
+    <row r="6" spans="1:22">
+      <c r="A6" s="4">
+        <v>45919</v>
+      </c>
       <c r="B6" s="8" t="s">
         <v>37</v>
       </c>
@@ -1086,8 +1115,8 @@
       <c r="K6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="9">
-        <v>4</v>
+      <c r="L6" s="4">
+        <v>45919</v>
       </c>
       <c r="M6" s="9">
         <v>4</v>
@@ -1101,23 +1130,26 @@
       <c r="P6" s="9">
         <v>4</v>
       </c>
-      <c r="Q6" s="4">
-        <v>45919</v>
-      </c>
-      <c r="R6" s="9">
+      <c r="Q6" s="9">
         <v>4</v>
       </c>
-      <c r="S6" s="4">
-        <v>45919</v>
-      </c>
-      <c r="T6" s="3" t="s">
+      <c r="R6" s="4">
+        <v>45919</v>
+      </c>
+      <c r="S6" s="9">
+        <v>4</v>
+      </c>
+      <c r="T6" s="4">
+        <v>45919</v>
+      </c>
+      <c r="U6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U6" s="8" t="s">
+      <c r="V6" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:22">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1126,10 +1158,10 @@
       <c r="F7" s="6"/>
       <c r="I7" s="6"/>
       <c r="J7" s="7"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="5"/>
-    </row>
-    <row r="8" spans="1:21">
+      <c r="Q7" s="6"/>
+      <c r="R7" s="5"/>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1138,10 +1170,10 @@
       <c r="F8" s="6"/>
       <c r="I8" s="6"/>
       <c r="J8" s="7"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="5"/>
-    </row>
-    <row r="9" spans="1:21">
+      <c r="Q8" s="6"/>
+      <c r="R8" s="5"/>
+    </row>
+    <row r="9" spans="1:22">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1150,10 +1182,10 @@
       <c r="F9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="7"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="5"/>
-    </row>
-    <row r="10" spans="1:21">
+      <c r="Q9" s="6"/>
+      <c r="R9" s="5"/>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1162,10 +1194,10 @@
       <c r="F10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="7"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="5"/>
-    </row>
-    <row r="11" spans="1:21">
+      <c r="Q10" s="6"/>
+      <c r="R10" s="5"/>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1174,10 +1206,10 @@
       <c r="F11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="7"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="5"/>
-    </row>
-    <row r="12" spans="1:21">
+      <c r="Q11" s="6"/>
+      <c r="R11" s="5"/>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1186,10 +1218,10 @@
       <c r="F12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="7"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="5"/>
-    </row>
-    <row r="13" spans="1:21">
+      <c r="Q12" s="6"/>
+      <c r="R12" s="5"/>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1198,10 +1230,10 @@
       <c r="F13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="7"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="5"/>
-    </row>
-    <row r="14" spans="1:21">
+      <c r="Q13" s="6"/>
+      <c r="R13" s="5"/>
+    </row>
+    <row r="14" spans="1:22">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1210,10 +1242,10 @@
       <c r="F14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="7"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="5"/>
-    </row>
-    <row r="15" spans="1:21">
+      <c r="Q14" s="6"/>
+      <c r="R14" s="5"/>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1222,10 +1254,10 @@
       <c r="F15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="7"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="5"/>
-    </row>
-    <row r="16" spans="1:21">
+      <c r="Q15" s="6"/>
+      <c r="R15" s="5"/>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1234,8 +1266,8 @@
       <c r="F16" s="6"/>
       <c r="I16" s="6"/>
       <c r="J16" s="7"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="5"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>